<commit_message>
feat: Add type field to StaffPromotion model and migration
- Introduced a new 'type' field in the StaffPromotion model to differentiate between 'promotion' and 'conversion'.
- Implemented a method to detect the type based on payroll number and salary structure.
- Updated the AuthServiceProvider to streamline permission checks using a mapping array.
- Refactored sidebar and layout views to conditionally display the sidebar for non-admin users.
- Enhanced employee promotion views to include the new 'type' field and updated titles accordingly.
- Added a new migration to include the 'type' column in the staff_promotions table.
</commit_message>
<xml_diff>
--- a/public/assets/excel_sample/promotion.xlsx
+++ b/public/assets/excel_sample/promotion.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Payroll\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE3CC8BA-E28A-4860-8731-900A7DE67E90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{570C813C-A30E-4A34-9597-C479252508E3}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12570"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="17">
   <si>
     <t>payroll_number</t>
   </si>
@@ -39,31 +38,49 @@
     <t>step</t>
   </si>
   <si>
-    <t>TI113216</t>
-  </si>
-  <si>
-    <t>TI131288</t>
-  </si>
-  <si>
-    <t>TI115090</t>
-  </si>
-  <si>
-    <t>TI131290</t>
-  </si>
-  <si>
-    <t>TI131292</t>
-  </si>
-  <si>
-    <t>CONTEDISS</t>
-  </si>
-  <si>
-    <t>COMPCASS</t>
+    <t>TI137104</t>
+  </si>
+  <si>
+    <t>TI137486</t>
+  </si>
+  <si>
+    <t>TI137118</t>
+  </si>
+  <si>
+    <t>TI137106</t>
+  </si>
+  <si>
+    <t>TI137117</t>
+  </si>
+  <si>
+    <t>CONUASS</t>
+  </si>
+  <si>
+    <t>TI135868</t>
+  </si>
+  <si>
+    <t>TI135870</t>
+  </si>
+  <si>
+    <t>TI135941</t>
+  </si>
+  <si>
+    <t>TI135942</t>
+  </si>
+  <si>
+    <t>TI137338</t>
+  </si>
+  <si>
+    <t>TI137332</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONTISS </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -408,16 +425,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{756D41D2-7523-4E79-981B-16BEC67BE94B}">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.6640625" customWidth="1"/>
-    <col min="2" max="2" width="26.44140625" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -431,7 +448,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -442,10 +459,10 @@
         <v>7</v>
       </c>
       <c r="D2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -453,13 +470,13 @@
         <v>9</v>
       </c>
       <c r="C3">
+        <v>7</v>
+      </c>
+      <c r="D3">
         <v>6</v>
       </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -467,27 +484,27 @@
         <v>9</v>
       </c>
       <c r="C4">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D4">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -495,10 +512,94 @@
         <v>9</v>
       </c>
       <c r="C6">
+        <v>7</v>
+      </c>
+      <c r="D6">
         <v>6</v>
       </c>
-      <c r="D6">
-        <v>1</v>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7">
+        <v>15</v>
+      </c>
+      <c r="D7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8">
+        <v>15</v>
+      </c>
+      <c r="D8">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9">
+        <v>15</v>
+      </c>
+      <c r="D9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10">
+        <v>15</v>
+      </c>
+      <c r="D10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11">
+        <v>15</v>
+      </c>
+      <c r="D11">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12">
+        <v>15</v>
+      </c>
+      <c r="D12">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>